<commit_message>
Agave Ridge concrete foundations CO 1 pricing (10/26/2026)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D6wjrb1spFgY1HgqZrWwPC
</commit_message>
<xml_diff>
--- a/TriPointeContracts1.xlsx
+++ b/TriPointeContracts1.xlsx
@@ -16,9 +16,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -49,10 +48,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G127"/>
+  <dimension ref="A1:G139"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -476,7 +476,7 @@
       <c r="B2" t="n">
         <v>1</v>
       </c>
-      <c r="C2" s="1" t="n">
+      <c r="C2" s="3" t="n">
         <v>46185</v>
       </c>
       <c r="D2" t="inlineStr">
@@ -492,7 +492,6 @@
       <c r="F2" s="2" t="n">
         <v>33459</v>
       </c>
-      <c r="G2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -503,7 +502,7 @@
       <c r="B3" t="n">
         <v>1</v>
       </c>
-      <c r="C3" s="1" t="n">
+      <c r="C3" s="3" t="n">
         <v>46185</v>
       </c>
       <c r="D3" t="inlineStr">
@@ -519,7 +518,6 @@
       <c r="F3" s="2" t="n">
         <v>33887</v>
       </c>
-      <c r="G3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -530,7 +528,7 @@
       <c r="B4" t="n">
         <v>1</v>
       </c>
-      <c r="C4" s="1" t="n">
+      <c r="C4" s="3" t="n">
         <v>46185</v>
       </c>
       <c r="D4" t="inlineStr">
@@ -546,7 +544,6 @@
       <c r="F4" s="2" t="n">
         <v>33459</v>
       </c>
-      <c r="G4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -557,7 +554,7 @@
       <c r="B5" t="n">
         <v>1</v>
       </c>
-      <c r="C5" s="1" t="n">
+      <c r="C5" s="3" t="n">
         <v>46185</v>
       </c>
       <c r="D5" t="inlineStr">
@@ -573,7 +570,6 @@
       <c r="F5" s="2" t="n">
         <v>34229</v>
       </c>
-      <c r="G5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -584,7 +580,7 @@
       <c r="B6" t="n">
         <v>1</v>
       </c>
-      <c r="C6" s="1" t="n">
+      <c r="C6" s="3" t="n">
         <v>46185</v>
       </c>
       <c r="D6" t="inlineStr">
@@ -600,7 +596,6 @@
       <c r="F6" s="2" t="n">
         <v>34520</v>
       </c>
-      <c r="G6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -611,7 +606,7 @@
       <c r="B7" t="n">
         <v>1</v>
       </c>
-      <c r="C7" s="1" t="n">
+      <c r="C7" s="3" t="n">
         <v>46185</v>
       </c>
       <c r="D7" t="inlineStr">
@@ -627,7 +622,6 @@
       <c r="F7" s="2" t="n">
         <v>34229</v>
       </c>
-      <c r="G7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -638,7 +632,7 @@
       <c r="B8" t="n">
         <v>1</v>
       </c>
-      <c r="C8" s="1" t="n">
+      <c r="C8" s="3" t="n">
         <v>46185</v>
       </c>
       <c r="D8" t="inlineStr">
@@ -654,7 +648,6 @@
       <c r="F8" s="2" t="n">
         <v>37234</v>
       </c>
-      <c r="G8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -665,7 +658,7 @@
       <c r="B9" t="n">
         <v>1</v>
       </c>
-      <c r="C9" s="1" t="n">
+      <c r="C9" s="3" t="n">
         <v>46185</v>
       </c>
       <c r="D9" t="inlineStr">
@@ -681,7 +674,6 @@
       <c r="F9" s="2" t="n">
         <v>37525</v>
       </c>
-      <c r="G9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -692,7 +684,7 @@
       <c r="B10" t="n">
         <v>1</v>
       </c>
-      <c r="C10" s="1" t="n">
+      <c r="C10" s="3" t="n">
         <v>46185</v>
       </c>
       <c r="D10" t="inlineStr">
@@ -708,7 +700,6 @@
       <c r="F10" s="2" t="n">
         <v>37234</v>
       </c>
-      <c r="G10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -719,7 +710,7 @@
       <c r="B11" t="n">
         <v>1</v>
       </c>
-      <c r="C11" s="1" t="n">
+      <c r="C11" s="3" t="n">
         <v>46185</v>
       </c>
       <c r="D11" t="inlineStr">
@@ -735,7 +726,6 @@
       <c r="F11" s="2" t="n">
         <v>39949</v>
       </c>
-      <c r="G11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -746,7 +736,7 @@
       <c r="B12" t="n">
         <v>1</v>
       </c>
-      <c r="C12" s="1" t="n">
+      <c r="C12" s="3" t="n">
         <v>46185</v>
       </c>
       <c r="D12" t="inlineStr">
@@ -762,7 +752,6 @@
       <c r="F12" s="2" t="n">
         <v>40398</v>
       </c>
-      <c r="G12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -773,7 +762,7 @@
       <c r="B13" t="n">
         <v>1</v>
       </c>
-      <c r="C13" s="1" t="n">
+      <c r="C13" s="3" t="n">
         <v>46185</v>
       </c>
       <c r="D13" t="inlineStr">
@@ -789,7 +778,6 @@
       <c r="F13" s="2" t="n">
         <v>39949</v>
       </c>
-      <c r="G13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -800,8 +788,8 @@
       <c r="B14" t="n">
         <v>1</v>
       </c>
-      <c r="C14" s="1" t="n">
-        <v>46185</v>
+      <c r="C14" s="3" t="n">
+        <v>46321</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -810,13 +798,17 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>FND-DROP 6"-12"</t>
+          <t>Foundation</t>
         </is>
       </c>
       <c r="F14" s="2" t="n">
-        <v>1916</v>
-      </c>
-      <c r="G14" t="inlineStr"/>
+        <v>33126</v>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>CO #1 - courtyard wall footings deleted</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -827,8 +819,8 @@
       <c r="B15" t="n">
         <v>1</v>
       </c>
-      <c r="C15" s="1" t="n">
-        <v>46185</v>
+      <c r="C15" s="3" t="n">
+        <v>46321</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -837,13 +829,17 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>FND-DROP 6"-12"</t>
+          <t>Foundation</t>
         </is>
       </c>
       <c r="F15" s="2" t="n">
-        <v>1916</v>
-      </c>
-      <c r="G15" t="inlineStr"/>
+        <v>33554</v>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>CO #1 - courtyard wall footings deleted</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -854,8 +850,8 @@
       <c r="B16" t="n">
         <v>1</v>
       </c>
-      <c r="C16" s="1" t="n">
-        <v>46185</v>
+      <c r="C16" s="3" t="n">
+        <v>46321</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -864,13 +860,17 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>FND-DROP 6"-12"</t>
+          <t>Foundation</t>
         </is>
       </c>
       <c r="F16" s="2" t="n">
-        <v>1916</v>
-      </c>
-      <c r="G16" t="inlineStr"/>
+        <v>33126</v>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>CO #1 - courtyard wall footings deleted</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -881,8 +881,8 @@
       <c r="B17" t="n">
         <v>1</v>
       </c>
-      <c r="C17" s="1" t="n">
-        <v>46185</v>
+      <c r="C17" s="3" t="n">
+        <v>46321</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -891,13 +891,17 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>FND-DROP 6"-12"</t>
+          <t>Foundation</t>
         </is>
       </c>
       <c r="F17" s="2" t="n">
-        <v>1916</v>
-      </c>
-      <c r="G17" t="inlineStr"/>
+        <v>33555</v>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>CO #1 - courtyard wall footings deleted</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -908,8 +912,8 @@
       <c r="B18" t="n">
         <v>1</v>
       </c>
-      <c r="C18" s="1" t="n">
-        <v>46185</v>
+      <c r="C18" s="3" t="n">
+        <v>46321</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -918,13 +922,17 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>FND-DROP 6"-12"</t>
+          <t>Foundation</t>
         </is>
       </c>
       <c r="F18" s="2" t="n">
-        <v>1916</v>
-      </c>
-      <c r="G18" t="inlineStr"/>
+        <v>33846</v>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>CO #1 - courtyard wall footings deleted</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -935,8 +943,8 @@
       <c r="B19" t="n">
         <v>1</v>
       </c>
-      <c r="C19" s="1" t="n">
-        <v>46185</v>
+      <c r="C19" s="3" t="n">
+        <v>46321</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -945,13 +953,17 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>FND-DROP 6"-12"</t>
+          <t>Foundation</t>
         </is>
       </c>
       <c r="F19" s="2" t="n">
-        <v>1916</v>
-      </c>
-      <c r="G19" t="inlineStr"/>
+        <v>33555</v>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>CO #1 - courtyard wall footings deleted</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -962,8 +974,8 @@
       <c r="B20" t="n">
         <v>1</v>
       </c>
-      <c r="C20" s="1" t="n">
-        <v>46185</v>
+      <c r="C20" s="3" t="n">
+        <v>46321</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -972,13 +984,17 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>FND-DROP 6"-12"</t>
+          <t>Foundation</t>
         </is>
       </c>
       <c r="F20" s="2" t="n">
-        <v>1916</v>
-      </c>
-      <c r="G20" t="inlineStr"/>
+        <v>37065</v>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>CO #1 - courtyard wall footings deleted</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -989,8 +1005,8 @@
       <c r="B21" t="n">
         <v>1</v>
       </c>
-      <c r="C21" s="1" t="n">
-        <v>46185</v>
+      <c r="C21" s="3" t="n">
+        <v>46321</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
@@ -999,13 +1015,17 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>FND-DROP 6"-12"</t>
+          <t>Foundation</t>
         </is>
       </c>
       <c r="F21" s="2" t="n">
-        <v>1916</v>
-      </c>
-      <c r="G21" t="inlineStr"/>
+        <v>37356</v>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>CO #1 - courtyard wall footings deleted</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1016,8 +1036,8 @@
       <c r="B22" t="n">
         <v>1</v>
       </c>
-      <c r="C22" s="1" t="n">
-        <v>46185</v>
+      <c r="C22" s="3" t="n">
+        <v>46321</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
@@ -1026,13 +1046,17 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>FND-DROP 6"-12"</t>
+          <t>Foundation</t>
         </is>
       </c>
       <c r="F22" s="2" t="n">
-        <v>1916</v>
-      </c>
-      <c r="G22" t="inlineStr"/>
+        <v>37065</v>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>CO #1 - courtyard wall footings deleted</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1043,8 +1067,8 @@
       <c r="B23" t="n">
         <v>1</v>
       </c>
-      <c r="C23" s="1" t="n">
-        <v>46185</v>
+      <c r="C23" s="3" t="n">
+        <v>46321</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
@@ -1053,13 +1077,17 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>FND-DROP 6"-12"</t>
+          <t>Foundation</t>
         </is>
       </c>
       <c r="F23" s="2" t="n">
-        <v>1916</v>
-      </c>
-      <c r="G23" t="inlineStr"/>
+        <v>39773</v>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>CO #1 - courtyard wall footings deleted</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1070,8 +1098,8 @@
       <c r="B24" t="n">
         <v>1</v>
       </c>
-      <c r="C24" s="1" t="n">
-        <v>46185</v>
+      <c r="C24" s="3" t="n">
+        <v>46321</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
@@ -1080,13 +1108,17 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>FND-DROP 6"-12"</t>
+          <t>Foundation</t>
         </is>
       </c>
       <c r="F24" s="2" t="n">
-        <v>1916</v>
-      </c>
-      <c r="G24" t="inlineStr"/>
+        <v>40222</v>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>CO #1 - courtyard wall footings deleted</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1097,8 +1129,8 @@
       <c r="B25" t="n">
         <v>1</v>
       </c>
-      <c r="C25" s="1" t="n">
-        <v>46185</v>
+      <c r="C25" s="3" t="n">
+        <v>46321</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
@@ -1107,13 +1139,17 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>FND-DROP 6"-12"</t>
+          <t>Foundation</t>
         </is>
       </c>
       <c r="F25" s="2" t="n">
-        <v>1916</v>
-      </c>
-      <c r="G25" t="inlineStr"/>
+        <v>39773</v>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>CO #1 - courtyard wall footings deleted</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1124,7 +1160,7 @@
       <c r="B26" t="n">
         <v>1</v>
       </c>
-      <c r="C26" s="1" t="n">
+      <c r="C26" s="3" t="n">
         <v>46185</v>
       </c>
       <c r="D26" t="inlineStr">
@@ -1134,13 +1170,12 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>FND-DROP 13"-18"</t>
+          <t>FND-DROP 6"-12"</t>
         </is>
       </c>
       <c r="F26" s="2" t="n">
-        <v>3757</v>
-      </c>
-      <c r="G26" t="inlineStr"/>
+        <v>1916</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1151,7 +1186,7 @@
       <c r="B27" t="n">
         <v>1</v>
       </c>
-      <c r="C27" s="1" t="n">
+      <c r="C27" s="3" t="n">
         <v>46185</v>
       </c>
       <c r="D27" t="inlineStr">
@@ -1161,13 +1196,12 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>FND-DROP 13"-18"</t>
+          <t>FND-DROP 6"-12"</t>
         </is>
       </c>
       <c r="F27" s="2" t="n">
-        <v>3757</v>
-      </c>
-      <c r="G27" t="inlineStr"/>
+        <v>1916</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1178,7 +1212,7 @@
       <c r="B28" t="n">
         <v>1</v>
       </c>
-      <c r="C28" s="1" t="n">
+      <c r="C28" s="3" t="n">
         <v>46185</v>
       </c>
       <c r="D28" t="inlineStr">
@@ -1188,13 +1222,12 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>FND-DROP 13"-18"</t>
+          <t>FND-DROP 6"-12"</t>
         </is>
       </c>
       <c r="F28" s="2" t="n">
-        <v>3757</v>
-      </c>
-      <c r="G28" t="inlineStr"/>
+        <v>1916</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1205,7 +1238,7 @@
       <c r="B29" t="n">
         <v>1</v>
       </c>
-      <c r="C29" s="1" t="n">
+      <c r="C29" s="3" t="n">
         <v>46185</v>
       </c>
       <c r="D29" t="inlineStr">
@@ -1215,13 +1248,12 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>FND-DROP 13"-18"</t>
+          <t>FND-DROP 6"-12"</t>
         </is>
       </c>
       <c r="F29" s="2" t="n">
-        <v>3757</v>
-      </c>
-      <c r="G29" t="inlineStr"/>
+        <v>1916</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1232,7 +1264,7 @@
       <c r="B30" t="n">
         <v>1</v>
       </c>
-      <c r="C30" s="1" t="n">
+      <c r="C30" s="3" t="n">
         <v>46185</v>
       </c>
       <c r="D30" t="inlineStr">
@@ -1242,13 +1274,12 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>FND-DROP 13"-18"</t>
+          <t>FND-DROP 6"-12"</t>
         </is>
       </c>
       <c r="F30" s="2" t="n">
-        <v>3757</v>
-      </c>
-      <c r="G30" t="inlineStr"/>
+        <v>1916</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1259,7 +1290,7 @@
       <c r="B31" t="n">
         <v>1</v>
       </c>
-      <c r="C31" s="1" t="n">
+      <c r="C31" s="3" t="n">
         <v>46185</v>
       </c>
       <c r="D31" t="inlineStr">
@@ -1269,13 +1300,12 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>FND-DROP 13"-18"</t>
+          <t>FND-DROP 6"-12"</t>
         </is>
       </c>
       <c r="F31" s="2" t="n">
-        <v>3757</v>
-      </c>
-      <c r="G31" t="inlineStr"/>
+        <v>1916</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1286,7 +1316,7 @@
       <c r="B32" t="n">
         <v>1</v>
       </c>
-      <c r="C32" s="1" t="n">
+      <c r="C32" s="3" t="n">
         <v>46185</v>
       </c>
       <c r="D32" t="inlineStr">
@@ -1296,13 +1326,12 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>FND-DROP 13"-18"</t>
+          <t>FND-DROP 6"-12"</t>
         </is>
       </c>
       <c r="F32" s="2" t="n">
-        <v>3757</v>
-      </c>
-      <c r="G32" t="inlineStr"/>
+        <v>1916</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1313,7 +1342,7 @@
       <c r="B33" t="n">
         <v>1</v>
       </c>
-      <c r="C33" s="1" t="n">
+      <c r="C33" s="3" t="n">
         <v>46185</v>
       </c>
       <c r="D33" t="inlineStr">
@@ -1323,13 +1352,12 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>FND-DROP 13"-18"</t>
+          <t>FND-DROP 6"-12"</t>
         </is>
       </c>
       <c r="F33" s="2" t="n">
-        <v>3757</v>
-      </c>
-      <c r="G33" t="inlineStr"/>
+        <v>1916</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1340,7 +1368,7 @@
       <c r="B34" t="n">
         <v>1</v>
       </c>
-      <c r="C34" s="1" t="n">
+      <c r="C34" s="3" t="n">
         <v>46185</v>
       </c>
       <c r="D34" t="inlineStr">
@@ -1350,13 +1378,12 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>FND-DROP 13"-18"</t>
+          <t>FND-DROP 6"-12"</t>
         </is>
       </c>
       <c r="F34" s="2" t="n">
-        <v>3757</v>
-      </c>
-      <c r="G34" t="inlineStr"/>
+        <v>1916</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1367,7 +1394,7 @@
       <c r="B35" t="n">
         <v>1</v>
       </c>
-      <c r="C35" s="1" t="n">
+      <c r="C35" s="3" t="n">
         <v>46185</v>
       </c>
       <c r="D35" t="inlineStr">
@@ -1377,13 +1404,12 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>FND-DROP 13"-18"</t>
+          <t>FND-DROP 6"-12"</t>
         </is>
       </c>
       <c r="F35" s="2" t="n">
-        <v>3757</v>
-      </c>
-      <c r="G35" t="inlineStr"/>
+        <v>1916</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1394,7 +1420,7 @@
       <c r="B36" t="n">
         <v>1</v>
       </c>
-      <c r="C36" s="1" t="n">
+      <c r="C36" s="3" t="n">
         <v>46185</v>
       </c>
       <c r="D36" t="inlineStr">
@@ -1404,13 +1430,12 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>FND-DROP 13"-18"</t>
+          <t>FND-DROP 6"-12"</t>
         </is>
       </c>
       <c r="F36" s="2" t="n">
-        <v>3757</v>
-      </c>
-      <c r="G36" t="inlineStr"/>
+        <v>1916</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1421,7 +1446,7 @@
       <c r="B37" t="n">
         <v>1</v>
       </c>
-      <c r="C37" s="1" t="n">
+      <c r="C37" s="3" t="n">
         <v>46185</v>
       </c>
       <c r="D37" t="inlineStr">
@@ -1431,13 +1456,12 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>FND-DROP 13"-18"</t>
+          <t>FND-DROP 6"-12"</t>
         </is>
       </c>
       <c r="F37" s="2" t="n">
-        <v>3757</v>
-      </c>
-      <c r="G37" t="inlineStr"/>
+        <v>1916</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1448,7 +1472,7 @@
       <c r="B38" t="n">
         <v>1</v>
       </c>
-      <c r="C38" s="1" t="n">
+      <c r="C38" s="3" t="n">
         <v>46185</v>
       </c>
       <c r="D38" t="inlineStr">
@@ -1458,13 +1482,12 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>FND-DROP 19"-24"</t>
+          <t>FND-DROP 13"-18"</t>
         </is>
       </c>
       <c r="F38" s="2" t="n">
-        <v>5598</v>
-      </c>
-      <c r="G38" t="inlineStr"/>
+        <v>3757</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1475,7 +1498,7 @@
       <c r="B39" t="n">
         <v>1</v>
       </c>
-      <c r="C39" s="1" t="n">
+      <c r="C39" s="3" t="n">
         <v>46185</v>
       </c>
       <c r="D39" t="inlineStr">
@@ -1485,13 +1508,12 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>FND-DROP 19"-24"</t>
+          <t>FND-DROP 13"-18"</t>
         </is>
       </c>
       <c r="F39" s="2" t="n">
-        <v>5598</v>
-      </c>
-      <c r="G39" t="inlineStr"/>
+        <v>3757</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -1502,7 +1524,7 @@
       <c r="B40" t="n">
         <v>1</v>
       </c>
-      <c r="C40" s="1" t="n">
+      <c r="C40" s="3" t="n">
         <v>46185</v>
       </c>
       <c r="D40" t="inlineStr">
@@ -1512,13 +1534,12 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>FND-DROP 19"-24"</t>
+          <t>FND-DROP 13"-18"</t>
         </is>
       </c>
       <c r="F40" s="2" t="n">
-        <v>5598</v>
-      </c>
-      <c r="G40" t="inlineStr"/>
+        <v>3757</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -1529,7 +1550,7 @@
       <c r="B41" t="n">
         <v>1</v>
       </c>
-      <c r="C41" s="1" t="n">
+      <c r="C41" s="3" t="n">
         <v>46185</v>
       </c>
       <c r="D41" t="inlineStr">
@@ -1539,13 +1560,12 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>FND-DROP 19"-24"</t>
+          <t>FND-DROP 13"-18"</t>
         </is>
       </c>
       <c r="F41" s="2" t="n">
-        <v>5598</v>
-      </c>
-      <c r="G41" t="inlineStr"/>
+        <v>3757</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -1556,7 +1576,7 @@
       <c r="B42" t="n">
         <v>1</v>
       </c>
-      <c r="C42" s="1" t="n">
+      <c r="C42" s="3" t="n">
         <v>46185</v>
       </c>
       <c r="D42" t="inlineStr">
@@ -1566,13 +1586,12 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>FND-DROP 19"-24"</t>
+          <t>FND-DROP 13"-18"</t>
         </is>
       </c>
       <c r="F42" s="2" t="n">
-        <v>5598</v>
-      </c>
-      <c r="G42" t="inlineStr"/>
+        <v>3757</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -1583,7 +1602,7 @@
       <c r="B43" t="n">
         <v>1</v>
       </c>
-      <c r="C43" s="1" t="n">
+      <c r="C43" s="3" t="n">
         <v>46185</v>
       </c>
       <c r="D43" t="inlineStr">
@@ -1593,13 +1612,12 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>FND-DROP 19"-24"</t>
+          <t>FND-DROP 13"-18"</t>
         </is>
       </c>
       <c r="F43" s="2" t="n">
-        <v>5598</v>
-      </c>
-      <c r="G43" t="inlineStr"/>
+        <v>3757</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -1610,7 +1628,7 @@
       <c r="B44" t="n">
         <v>1</v>
       </c>
-      <c r="C44" s="1" t="n">
+      <c r="C44" s="3" t="n">
         <v>46185</v>
       </c>
       <c r="D44" t="inlineStr">
@@ -1620,13 +1638,12 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>FND-DROP 19"-24"</t>
+          <t>FND-DROP 13"-18"</t>
         </is>
       </c>
       <c r="F44" s="2" t="n">
-        <v>5598</v>
-      </c>
-      <c r="G44" t="inlineStr"/>
+        <v>3757</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -1637,7 +1654,7 @@
       <c r="B45" t="n">
         <v>1</v>
       </c>
-      <c r="C45" s="1" t="n">
+      <c r="C45" s="3" t="n">
         <v>46185</v>
       </c>
       <c r="D45" t="inlineStr">
@@ -1647,13 +1664,12 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>FND-DROP 19"-24"</t>
+          <t>FND-DROP 13"-18"</t>
         </is>
       </c>
       <c r="F45" s="2" t="n">
-        <v>5598</v>
-      </c>
-      <c r="G45" t="inlineStr"/>
+        <v>3757</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -1664,7 +1680,7 @@
       <c r="B46" t="n">
         <v>1</v>
       </c>
-      <c r="C46" s="1" t="n">
+      <c r="C46" s="3" t="n">
         <v>46185</v>
       </c>
       <c r="D46" t="inlineStr">
@@ -1674,13 +1690,12 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>FND-DROP 19"-24"</t>
+          <t>FND-DROP 13"-18"</t>
         </is>
       </c>
       <c r="F46" s="2" t="n">
-        <v>5598</v>
-      </c>
-      <c r="G46" t="inlineStr"/>
+        <v>3757</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -1691,7 +1706,7 @@
       <c r="B47" t="n">
         <v>1</v>
       </c>
-      <c r="C47" s="1" t="n">
+      <c r="C47" s="3" t="n">
         <v>46185</v>
       </c>
       <c r="D47" t="inlineStr">
@@ -1701,13 +1716,12 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>FND-DROP 19"-24"</t>
+          <t>FND-DROP 13"-18"</t>
         </is>
       </c>
       <c r="F47" s="2" t="n">
-        <v>5598</v>
-      </c>
-      <c r="G47" t="inlineStr"/>
+        <v>3757</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -1718,7 +1732,7 @@
       <c r="B48" t="n">
         <v>1</v>
       </c>
-      <c r="C48" s="1" t="n">
+      <c r="C48" s="3" t="n">
         <v>46185</v>
       </c>
       <c r="D48" t="inlineStr">
@@ -1728,13 +1742,12 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>FND-DROP 19"-24"</t>
+          <t>FND-DROP 13"-18"</t>
         </is>
       </c>
       <c r="F48" s="2" t="n">
-        <v>5598</v>
-      </c>
-      <c r="G48" t="inlineStr"/>
+        <v>3757</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -1745,7 +1758,7 @@
       <c r="B49" t="n">
         <v>1</v>
       </c>
-      <c r="C49" s="1" t="n">
+      <c r="C49" s="3" t="n">
         <v>46185</v>
       </c>
       <c r="D49" t="inlineStr">
@@ -1755,25 +1768,24 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>FND-DROP 19"-24"</t>
+          <t>FND-DROP 13"-18"</t>
         </is>
       </c>
       <c r="F49" s="2" t="n">
-        <v>5598</v>
-      </c>
-      <c r="G49" t="inlineStr"/>
+        <v>3757</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Edgewood - Concrete</t>
+          <t>Agave Ridge - Concrete</t>
         </is>
       </c>
       <c r="B50" t="n">
         <v>1</v>
       </c>
-      <c r="C50" s="1" t="n">
-        <v>45349</v>
+      <c r="C50" s="3" t="n">
+        <v>46185</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
@@ -1782,310 +1794,298 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Foundation</t>
+          <t>FND-DROP 19"-24"</t>
         </is>
       </c>
       <c r="F50" s="2" t="n">
-        <v>22656</v>
-      </c>
-      <c r="G50" t="inlineStr"/>
+        <v>5598</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Edgewood - Concrete</t>
+          <t>Agave Ridge - Concrete</t>
         </is>
       </c>
       <c r="B51" t="n">
         <v>1</v>
       </c>
-      <c r="C51" s="1" t="n">
-        <v>45349</v>
+      <c r="C51" s="3" t="n">
+        <v>46185</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Plan 2A</t>
+          <t>Plan 1B</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Foundation</t>
+          <t>FND-DROP 19"-24"</t>
         </is>
       </c>
       <c r="F51" s="2" t="n">
-        <v>24093</v>
-      </c>
-      <c r="G51" t="inlineStr"/>
+        <v>5598</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Edgewood - Concrete</t>
+          <t>Agave Ridge - Concrete</t>
         </is>
       </c>
       <c r="B52" t="n">
         <v>1</v>
       </c>
-      <c r="C52" s="1" t="n">
-        <v>45349</v>
+      <c r="C52" s="3" t="n">
+        <v>46185</v>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Plan 3A</t>
+          <t>Plan 1C</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Foundation</t>
+          <t>FND-DROP 19"-24"</t>
         </is>
       </c>
       <c r="F52" s="2" t="n">
-        <v>19990</v>
-      </c>
-      <c r="G52" t="inlineStr"/>
+        <v>5598</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Edgewood - Concrete</t>
+          <t>Agave Ridge - Concrete</t>
         </is>
       </c>
       <c r="B53" t="n">
         <v>1</v>
       </c>
-      <c r="C53" s="1" t="n">
-        <v>45349</v>
+      <c r="C53" s="3" t="n">
+        <v>46185</v>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Plan 4A</t>
+          <t>Plan 2A</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Foundation</t>
+          <t>FND-DROP 19"-24"</t>
         </is>
       </c>
       <c r="F53" s="2" t="n">
-        <v>21136</v>
-      </c>
-      <c r="G53" t="inlineStr"/>
+        <v>5598</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Edgewood - Concrete</t>
+          <t>Agave Ridge - Concrete</t>
         </is>
       </c>
       <c r="B54" t="n">
         <v>1</v>
       </c>
-      <c r="C54" s="1" t="n">
-        <v>45559</v>
+      <c r="C54" s="3" t="n">
+        <v>46185</v>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Plan 1A</t>
+          <t>Plan 2B</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Foundation</t>
+          <t>FND-DROP 19"-24"</t>
         </is>
       </c>
       <c r="F54" s="2" t="n">
-        <v>22656</v>
-      </c>
-      <c r="G54" t="inlineStr"/>
+        <v>5598</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Edgewood - Concrete</t>
+          <t>Agave Ridge - Concrete</t>
         </is>
       </c>
       <c r="B55" t="n">
         <v>1</v>
       </c>
-      <c r="C55" s="1" t="n">
-        <v>45559</v>
+      <c r="C55" s="3" t="n">
+        <v>46185</v>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Plan 1B</t>
+          <t>Plan 2C</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Foundation</t>
+          <t>FND-DROP 19"-24"</t>
         </is>
       </c>
       <c r="F55" s="2" t="n">
-        <v>24105</v>
-      </c>
-      <c r="G55" t="inlineStr"/>
+        <v>5598</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Edgewood - Concrete</t>
+          <t>Agave Ridge - Concrete</t>
         </is>
       </c>
       <c r="B56" t="n">
         <v>1</v>
       </c>
-      <c r="C56" s="1" t="n">
-        <v>45559</v>
+      <c r="C56" s="3" t="n">
+        <v>46185</v>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Plan 1C</t>
+          <t>Plan 3A</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Foundation</t>
+          <t>FND-DROP 19"-24"</t>
         </is>
       </c>
       <c r="F56" s="2" t="n">
-        <v>24651</v>
-      </c>
-      <c r="G56" t="inlineStr"/>
+        <v>5598</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Edgewood - Concrete</t>
+          <t>Agave Ridge - Concrete</t>
         </is>
       </c>
       <c r="B57" t="n">
         <v>1</v>
       </c>
-      <c r="C57" s="1" t="n">
-        <v>45559</v>
+      <c r="C57" s="3" t="n">
+        <v>46185</v>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Plan 2A</t>
+          <t>Plan 3B</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Foundation</t>
+          <t>FND-DROP 19"-24"</t>
         </is>
       </c>
       <c r="F57" s="2" t="n">
-        <v>24093</v>
-      </c>
-      <c r="G57" t="inlineStr"/>
+        <v>5598</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Edgewood - Concrete</t>
+          <t>Agave Ridge - Concrete</t>
         </is>
       </c>
       <c r="B58" t="n">
         <v>1</v>
       </c>
-      <c r="C58" s="1" t="n">
-        <v>45559</v>
+      <c r="C58" s="3" t="n">
+        <v>46185</v>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Plan 2B</t>
+          <t>Plan 3C</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Foundation</t>
+          <t>FND-DROP 19"-24"</t>
         </is>
       </c>
       <c r="F58" s="2" t="n">
-        <v>25989</v>
-      </c>
-      <c r="G58" t="inlineStr"/>
+        <v>5598</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Edgewood - Concrete</t>
+          <t>Agave Ridge - Concrete</t>
         </is>
       </c>
       <c r="B59" t="n">
         <v>1</v>
       </c>
-      <c r="C59" s="1" t="n">
-        <v>45559</v>
+      <c r="C59" s="3" t="n">
+        <v>46185</v>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Plan 2C</t>
+          <t>Plan 4A</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Foundation</t>
+          <t>FND-DROP 19"-24"</t>
         </is>
       </c>
       <c r="F59" s="2" t="n">
-        <v>26996</v>
-      </c>
-      <c r="G59" t="inlineStr"/>
+        <v>5598</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Edgewood - Concrete</t>
+          <t>Agave Ridge - Concrete</t>
         </is>
       </c>
       <c r="B60" t="n">
         <v>1</v>
       </c>
-      <c r="C60" s="1" t="n">
-        <v>45559</v>
+      <c r="C60" s="3" t="n">
+        <v>46185</v>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Plan 3A</t>
+          <t>Plan 4B</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Foundation</t>
+          <t>FND-DROP 19"-24"</t>
         </is>
       </c>
       <c r="F60" s="2" t="n">
-        <v>19990</v>
-      </c>
-      <c r="G60" t="inlineStr"/>
+        <v>5598</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Edgewood - Concrete</t>
+          <t>Agave Ridge - Concrete</t>
         </is>
       </c>
       <c r="B61" t="n">
         <v>1</v>
       </c>
-      <c r="C61" s="1" t="n">
-        <v>45559</v>
+      <c r="C61" s="3" t="n">
+        <v>46185</v>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Plan 3B</t>
+          <t>Plan 4C</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Foundation</t>
+          <t>FND-DROP 19"-24"</t>
         </is>
       </c>
       <c r="F61" s="2" t="n">
-        <v>19990</v>
-      </c>
-      <c r="G61" t="inlineStr"/>
+        <v>5598</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -2096,12 +2096,12 @@
       <c r="B62" t="n">
         <v>1</v>
       </c>
-      <c r="C62" s="1" t="n">
-        <v>45559</v>
+      <c r="C62" s="3" t="n">
+        <v>45349</v>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Plan 3C</t>
+          <t>Plan 1A</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
@@ -2110,9 +2110,8 @@
         </is>
       </c>
       <c r="F62" s="2" t="n">
-        <v>19990</v>
-      </c>
-      <c r="G62" t="inlineStr"/>
+        <v>22656</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -2123,12 +2122,12 @@
       <c r="B63" t="n">
         <v>1</v>
       </c>
-      <c r="C63" s="1" t="n">
-        <v>45559</v>
+      <c r="C63" s="3" t="n">
+        <v>45349</v>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Plan 4A</t>
+          <t>Plan 2A</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
@@ -2137,9 +2136,8 @@
         </is>
       </c>
       <c r="F63" s="2" t="n">
-        <v>21136</v>
-      </c>
-      <c r="G63" t="inlineStr"/>
+        <v>24093</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -2150,12 +2148,12 @@
       <c r="B64" t="n">
         <v>1</v>
       </c>
-      <c r="C64" s="1" t="n">
-        <v>45559</v>
+      <c r="C64" s="3" t="n">
+        <v>45349</v>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Plan 4B</t>
+          <t>Plan 3A</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
@@ -2164,9 +2162,8 @@
         </is>
       </c>
       <c r="F64" s="2" t="n">
-        <v>21568</v>
-      </c>
-      <c r="G64" t="inlineStr"/>
+        <v>19990</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -2177,12 +2174,12 @@
       <c r="B65" t="n">
         <v>1</v>
       </c>
-      <c r="C65" s="1" t="n">
-        <v>45559</v>
+      <c r="C65" s="3" t="n">
+        <v>45349</v>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Plan 4C</t>
+          <t>Plan 4A</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
@@ -2191,9 +2188,8 @@
         </is>
       </c>
       <c r="F65" s="2" t="n">
-        <v>21568</v>
-      </c>
-      <c r="G65" t="inlineStr"/>
+        <v>21136</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -2204,7 +2200,7 @@
       <c r="B66" t="n">
         <v>1</v>
       </c>
-      <c r="C66" s="1" t="n">
+      <c r="C66" s="3" t="n">
         <v>45559</v>
       </c>
       <c r="D66" t="inlineStr">
@@ -2214,13 +2210,12 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>FND-DROP 6"-12"</t>
+          <t>Foundation</t>
         </is>
       </c>
       <c r="F66" s="2" t="n">
-        <v>1174.25</v>
-      </c>
-      <c r="G66" t="inlineStr"/>
+        <v>22656</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -2231,7 +2226,7 @@
       <c r="B67" t="n">
         <v>1</v>
       </c>
-      <c r="C67" s="1" t="n">
+      <c r="C67" s="3" t="n">
         <v>45559</v>
       </c>
       <c r="D67" t="inlineStr">
@@ -2241,13 +2236,12 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>FND-DROP 6"-12"</t>
+          <t>Foundation</t>
         </is>
       </c>
       <c r="F67" s="2" t="n">
-        <v>1174.25</v>
-      </c>
-      <c r="G67" t="inlineStr"/>
+        <v>24105</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -2258,7 +2252,7 @@
       <c r="B68" t="n">
         <v>1</v>
       </c>
-      <c r="C68" s="1" t="n">
+      <c r="C68" s="3" t="n">
         <v>45559</v>
       </c>
       <c r="D68" t="inlineStr">
@@ -2268,13 +2262,12 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>FND-DROP 6"-12"</t>
+          <t>Foundation</t>
         </is>
       </c>
       <c r="F68" s="2" t="n">
-        <v>1174.25</v>
-      </c>
-      <c r="G68" t="inlineStr"/>
+        <v>24651</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -2285,7 +2278,7 @@
       <c r="B69" t="n">
         <v>1</v>
       </c>
-      <c r="C69" s="1" t="n">
+      <c r="C69" s="3" t="n">
         <v>45559</v>
       </c>
       <c r="D69" t="inlineStr">
@@ -2295,13 +2288,12 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>FND-DROP 6"-12"</t>
+          <t>Foundation</t>
         </is>
       </c>
       <c r="F69" s="2" t="n">
-        <v>1174.25</v>
-      </c>
-      <c r="G69" t="inlineStr"/>
+        <v>24093</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -2312,7 +2304,7 @@
       <c r="B70" t="n">
         <v>1</v>
       </c>
-      <c r="C70" s="1" t="n">
+      <c r="C70" s="3" t="n">
         <v>45559</v>
       </c>
       <c r="D70" t="inlineStr">
@@ -2322,13 +2314,12 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>FND-DROP 6"-12"</t>
+          <t>Foundation</t>
         </is>
       </c>
       <c r="F70" s="2" t="n">
-        <v>1174.25</v>
-      </c>
-      <c r="G70" t="inlineStr"/>
+        <v>25989</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -2339,7 +2330,7 @@
       <c r="B71" t="n">
         <v>1</v>
       </c>
-      <c r="C71" s="1" t="n">
+      <c r="C71" s="3" t="n">
         <v>45559</v>
       </c>
       <c r="D71" t="inlineStr">
@@ -2349,13 +2340,12 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>FND-DROP 6"-12"</t>
+          <t>Foundation</t>
         </is>
       </c>
       <c r="F71" s="2" t="n">
-        <v>1174.25</v>
-      </c>
-      <c r="G71" t="inlineStr"/>
+        <v>26996</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -2366,7 +2356,7 @@
       <c r="B72" t="n">
         <v>1</v>
       </c>
-      <c r="C72" s="1" t="n">
+      <c r="C72" s="3" t="n">
         <v>45559</v>
       </c>
       <c r="D72" t="inlineStr">
@@ -2376,13 +2366,12 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>FND-DROP 6"-12"</t>
+          <t>Foundation</t>
         </is>
       </c>
       <c r="F72" s="2" t="n">
-        <v>1174.25</v>
-      </c>
-      <c r="G72" t="inlineStr"/>
+        <v>19990</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -2393,7 +2382,7 @@
       <c r="B73" t="n">
         <v>1</v>
       </c>
-      <c r="C73" s="1" t="n">
+      <c r="C73" s="3" t="n">
         <v>45559</v>
       </c>
       <c r="D73" t="inlineStr">
@@ -2403,13 +2392,12 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>FND-DROP 6"-12"</t>
+          <t>Foundation</t>
         </is>
       </c>
       <c r="F73" s="2" t="n">
-        <v>1174.25</v>
-      </c>
-      <c r="G73" t="inlineStr"/>
+        <v>19990</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -2420,7 +2408,7 @@
       <c r="B74" t="n">
         <v>1</v>
       </c>
-      <c r="C74" s="1" t="n">
+      <c r="C74" s="3" t="n">
         <v>45559</v>
       </c>
       <c r="D74" t="inlineStr">
@@ -2430,13 +2418,12 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>FND-DROP 6"-12"</t>
+          <t>Foundation</t>
         </is>
       </c>
       <c r="F74" s="2" t="n">
-        <v>1174.25</v>
-      </c>
-      <c r="G74" t="inlineStr"/>
+        <v>19990</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -2447,7 +2434,7 @@
       <c r="B75" t="n">
         <v>1</v>
       </c>
-      <c r="C75" s="1" t="n">
+      <c r="C75" s="3" t="n">
         <v>45559</v>
       </c>
       <c r="D75" t="inlineStr">
@@ -2457,13 +2444,12 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>FND-DROP 6"-12"</t>
+          <t>Foundation</t>
         </is>
       </c>
       <c r="F75" s="2" t="n">
-        <v>1174.25</v>
-      </c>
-      <c r="G75" t="inlineStr"/>
+        <v>21136</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -2474,7 +2460,7 @@
       <c r="B76" t="n">
         <v>1</v>
       </c>
-      <c r="C76" s="1" t="n">
+      <c r="C76" s="3" t="n">
         <v>45559</v>
       </c>
       <c r="D76" t="inlineStr">
@@ -2484,13 +2470,12 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>FND-DROP 6"-12"</t>
+          <t>Foundation</t>
         </is>
       </c>
       <c r="F76" s="2" t="n">
-        <v>1174.25</v>
-      </c>
-      <c r="G76" t="inlineStr"/>
+        <v>21568</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -2501,7 +2486,7 @@
       <c r="B77" t="n">
         <v>1</v>
       </c>
-      <c r="C77" s="1" t="n">
+      <c r="C77" s="3" t="n">
         <v>45559</v>
       </c>
       <c r="D77" t="inlineStr">
@@ -2511,13 +2496,12 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>FND-DROP 6"-12"</t>
+          <t>Foundation</t>
         </is>
       </c>
       <c r="F77" s="2" t="n">
-        <v>1174.25</v>
-      </c>
-      <c r="G77" t="inlineStr"/>
+        <v>21568</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -2528,7 +2512,7 @@
       <c r="B78" t="n">
         <v>1</v>
       </c>
-      <c r="C78" s="1" t="n">
+      <c r="C78" s="3" t="n">
         <v>45559</v>
       </c>
       <c r="D78" t="inlineStr">
@@ -2538,13 +2522,12 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>FND-DROP 13"-18"</t>
+          <t>FND-DROP 6"-12"</t>
         </is>
       </c>
       <c r="F78" s="2" t="n">
-        <v>2303.25</v>
-      </c>
-      <c r="G78" t="inlineStr"/>
+        <v>1174.25</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -2555,7 +2538,7 @@
       <c r="B79" t="n">
         <v>1</v>
       </c>
-      <c r="C79" s="1" t="n">
+      <c r="C79" s="3" t="n">
         <v>45559</v>
       </c>
       <c r="D79" t="inlineStr">
@@ -2565,13 +2548,12 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>FND-DROP 13"-18"</t>
+          <t>FND-DROP 6"-12"</t>
         </is>
       </c>
       <c r="F79" s="2" t="n">
-        <v>2303.25</v>
-      </c>
-      <c r="G79" t="inlineStr"/>
+        <v>1174.25</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -2582,7 +2564,7 @@
       <c r="B80" t="n">
         <v>1</v>
       </c>
-      <c r="C80" s="1" t="n">
+      <c r="C80" s="3" t="n">
         <v>45559</v>
       </c>
       <c r="D80" t="inlineStr">
@@ -2592,13 +2574,12 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>FND-DROP 13"-18"</t>
+          <t>FND-DROP 6"-12"</t>
         </is>
       </c>
       <c r="F80" s="2" t="n">
-        <v>2303.25</v>
-      </c>
-      <c r="G80" t="inlineStr"/>
+        <v>1174.25</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -2609,7 +2590,7 @@
       <c r="B81" t="n">
         <v>1</v>
       </c>
-      <c r="C81" s="1" t="n">
+      <c r="C81" s="3" t="n">
         <v>45559</v>
       </c>
       <c r="D81" t="inlineStr">
@@ -2619,13 +2600,12 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>FND-DROP 13"-18"</t>
+          <t>FND-DROP 6"-12"</t>
         </is>
       </c>
       <c r="F81" s="2" t="n">
-        <v>2303.25</v>
-      </c>
-      <c r="G81" t="inlineStr"/>
+        <v>1174.25</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -2636,7 +2616,7 @@
       <c r="B82" t="n">
         <v>1</v>
       </c>
-      <c r="C82" s="1" t="n">
+      <c r="C82" s="3" t="n">
         <v>45559</v>
       </c>
       <c r="D82" t="inlineStr">
@@ -2646,13 +2626,12 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>FND-DROP 13"-18"</t>
+          <t>FND-DROP 6"-12"</t>
         </is>
       </c>
       <c r="F82" s="2" t="n">
-        <v>2303.25</v>
-      </c>
-      <c r="G82" t="inlineStr"/>
+        <v>1174.25</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -2663,7 +2642,7 @@
       <c r="B83" t="n">
         <v>1</v>
       </c>
-      <c r="C83" s="1" t="n">
+      <c r="C83" s="3" t="n">
         <v>45559</v>
       </c>
       <c r="D83" t="inlineStr">
@@ -2673,13 +2652,12 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>FND-DROP 13"-18"</t>
+          <t>FND-DROP 6"-12"</t>
         </is>
       </c>
       <c r="F83" s="2" t="n">
-        <v>2303.25</v>
-      </c>
-      <c r="G83" t="inlineStr"/>
+        <v>1174.25</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -2690,7 +2668,7 @@
       <c r="B84" t="n">
         <v>1</v>
       </c>
-      <c r="C84" s="1" t="n">
+      <c r="C84" s="3" t="n">
         <v>45559</v>
       </c>
       <c r="D84" t="inlineStr">
@@ -2700,13 +2678,12 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>FND-DROP 13"-18"</t>
+          <t>FND-DROP 6"-12"</t>
         </is>
       </c>
       <c r="F84" s="2" t="n">
-        <v>2303.25</v>
-      </c>
-      <c r="G84" t="inlineStr"/>
+        <v>1174.25</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -2717,7 +2694,7 @@
       <c r="B85" t="n">
         <v>1</v>
       </c>
-      <c r="C85" s="1" t="n">
+      <c r="C85" s="3" t="n">
         <v>45559</v>
       </c>
       <c r="D85" t="inlineStr">
@@ -2727,13 +2704,12 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>FND-DROP 13"-18"</t>
+          <t>FND-DROP 6"-12"</t>
         </is>
       </c>
       <c r="F85" s="2" t="n">
-        <v>2303.25</v>
-      </c>
-      <c r="G85" t="inlineStr"/>
+        <v>1174.25</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -2744,7 +2720,7 @@
       <c r="B86" t="n">
         <v>1</v>
       </c>
-      <c r="C86" s="1" t="n">
+      <c r="C86" s="3" t="n">
         <v>45559</v>
       </c>
       <c r="D86" t="inlineStr">
@@ -2754,13 +2730,12 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>FND-DROP 13"-18"</t>
+          <t>FND-DROP 6"-12"</t>
         </is>
       </c>
       <c r="F86" s="2" t="n">
-        <v>2303.25</v>
-      </c>
-      <c r="G86" t="inlineStr"/>
+        <v>1174.25</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -2771,7 +2746,7 @@
       <c r="B87" t="n">
         <v>1</v>
       </c>
-      <c r="C87" s="1" t="n">
+      <c r="C87" s="3" t="n">
         <v>45559</v>
       </c>
       <c r="D87" t="inlineStr">
@@ -2781,13 +2756,12 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>FND-DROP 13"-18"</t>
+          <t>FND-DROP 6"-12"</t>
         </is>
       </c>
       <c r="F87" s="2" t="n">
-        <v>2303.25</v>
-      </c>
-      <c r="G87" t="inlineStr"/>
+        <v>1174.25</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -2798,7 +2772,7 @@
       <c r="B88" t="n">
         <v>1</v>
       </c>
-      <c r="C88" s="1" t="n">
+      <c r="C88" s="3" t="n">
         <v>45559</v>
       </c>
       <c r="D88" t="inlineStr">
@@ -2808,13 +2782,12 @@
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>FND-DROP 13"-18"</t>
+          <t>FND-DROP 6"-12"</t>
         </is>
       </c>
       <c r="F88" s="2" t="n">
-        <v>2303.25</v>
-      </c>
-      <c r="G88" t="inlineStr"/>
+        <v>1174.25</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -2825,7 +2798,7 @@
       <c r="B89" t="n">
         <v>1</v>
       </c>
-      <c r="C89" s="1" t="n">
+      <c r="C89" s="3" t="n">
         <v>45559</v>
       </c>
       <c r="D89" t="inlineStr">
@@ -2835,13 +2808,12 @@
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>FND-DROP 13"-18"</t>
+          <t>FND-DROP 6"-12"</t>
         </is>
       </c>
       <c r="F89" s="2" t="n">
-        <v>2303.25</v>
-      </c>
-      <c r="G89" t="inlineStr"/>
+        <v>1174.25</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -2852,7 +2824,7 @@
       <c r="B90" t="n">
         <v>1</v>
       </c>
-      <c r="C90" s="1" t="n">
+      <c r="C90" s="3" t="n">
         <v>45559</v>
       </c>
       <c r="D90" t="inlineStr">
@@ -2862,13 +2834,12 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>FND-DROP 19"-24"</t>
+          <t>FND-DROP 13"-18"</t>
         </is>
       </c>
       <c r="F90" s="2" t="n">
-        <v>3432.5</v>
-      </c>
-      <c r="G90" t="inlineStr"/>
+        <v>2303.25</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -2879,7 +2850,7 @@
       <c r="B91" t="n">
         <v>1</v>
       </c>
-      <c r="C91" s="1" t="n">
+      <c r="C91" s="3" t="n">
         <v>45559</v>
       </c>
       <c r="D91" t="inlineStr">
@@ -2889,13 +2860,12 @@
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>FND-DROP 19"-24"</t>
+          <t>FND-DROP 13"-18"</t>
         </is>
       </c>
       <c r="F91" s="2" t="n">
-        <v>3432.5</v>
-      </c>
-      <c r="G91" t="inlineStr"/>
+        <v>2303.25</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -2906,7 +2876,7 @@
       <c r="B92" t="n">
         <v>1</v>
       </c>
-      <c r="C92" s="1" t="n">
+      <c r="C92" s="3" t="n">
         <v>45559</v>
       </c>
       <c r="D92" t="inlineStr">
@@ -2916,13 +2886,12 @@
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>FND-DROP 19"-24"</t>
+          <t>FND-DROP 13"-18"</t>
         </is>
       </c>
       <c r="F92" s="2" t="n">
-        <v>3432.5</v>
-      </c>
-      <c r="G92" t="inlineStr"/>
+        <v>2303.25</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -2933,7 +2902,7 @@
       <c r="B93" t="n">
         <v>1</v>
       </c>
-      <c r="C93" s="1" t="n">
+      <c r="C93" s="3" t="n">
         <v>45559</v>
       </c>
       <c r="D93" t="inlineStr">
@@ -2943,13 +2912,12 @@
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>FND-DROP 19"-24"</t>
+          <t>FND-DROP 13"-18"</t>
         </is>
       </c>
       <c r="F93" s="2" t="n">
-        <v>3432.5</v>
-      </c>
-      <c r="G93" t="inlineStr"/>
+        <v>2303.25</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -2960,7 +2928,7 @@
       <c r="B94" t="n">
         <v>1</v>
       </c>
-      <c r="C94" s="1" t="n">
+      <c r="C94" s="3" t="n">
         <v>45559</v>
       </c>
       <c r="D94" t="inlineStr">
@@ -2970,13 +2938,12 @@
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>FND-DROP 19"-24"</t>
+          <t>FND-DROP 13"-18"</t>
         </is>
       </c>
       <c r="F94" s="2" t="n">
-        <v>3432.5</v>
-      </c>
-      <c r="G94" t="inlineStr"/>
+        <v>2303.25</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -2987,7 +2954,7 @@
       <c r="B95" t="n">
         <v>1</v>
       </c>
-      <c r="C95" s="1" t="n">
+      <c r="C95" s="3" t="n">
         <v>45559</v>
       </c>
       <c r="D95" t="inlineStr">
@@ -2997,13 +2964,12 @@
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>FND-DROP 19"-24"</t>
+          <t>FND-DROP 13"-18"</t>
         </is>
       </c>
       <c r="F95" s="2" t="n">
-        <v>3432.5</v>
-      </c>
-      <c r="G95" t="inlineStr"/>
+        <v>2303.25</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -3014,7 +2980,7 @@
       <c r="B96" t="n">
         <v>1</v>
       </c>
-      <c r="C96" s="1" t="n">
+      <c r="C96" s="3" t="n">
         <v>45559</v>
       </c>
       <c r="D96" t="inlineStr">
@@ -3024,13 +2990,12 @@
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>FND-DROP 19"-24"</t>
+          <t>FND-DROP 13"-18"</t>
         </is>
       </c>
       <c r="F96" s="2" t="n">
-        <v>3432.5</v>
-      </c>
-      <c r="G96" t="inlineStr"/>
+        <v>2303.25</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -3041,7 +3006,7 @@
       <c r="B97" t="n">
         <v>1</v>
       </c>
-      <c r="C97" s="1" t="n">
+      <c r="C97" s="3" t="n">
         <v>45559</v>
       </c>
       <c r="D97" t="inlineStr">
@@ -3051,13 +3016,12 @@
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>FND-DROP 19"-24"</t>
+          <t>FND-DROP 13"-18"</t>
         </is>
       </c>
       <c r="F97" s="2" t="n">
-        <v>3432.5</v>
-      </c>
-      <c r="G97" t="inlineStr"/>
+        <v>2303.25</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -3068,7 +3032,7 @@
       <c r="B98" t="n">
         <v>1</v>
       </c>
-      <c r="C98" s="1" t="n">
+      <c r="C98" s="3" t="n">
         <v>45559</v>
       </c>
       <c r="D98" t="inlineStr">
@@ -3078,13 +3042,12 @@
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>FND-DROP 19"-24"</t>
+          <t>FND-DROP 13"-18"</t>
         </is>
       </c>
       <c r="F98" s="2" t="n">
-        <v>3432.5</v>
-      </c>
-      <c r="G98" t="inlineStr"/>
+        <v>2303.25</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -3095,7 +3058,7 @@
       <c r="B99" t="n">
         <v>1</v>
       </c>
-      <c r="C99" s="1" t="n">
+      <c r="C99" s="3" t="n">
         <v>45559</v>
       </c>
       <c r="D99" t="inlineStr">
@@ -3105,13 +3068,12 @@
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>FND-DROP 19"-24"</t>
+          <t>FND-DROP 13"-18"</t>
         </is>
       </c>
       <c r="F99" s="2" t="n">
-        <v>3432.5</v>
-      </c>
-      <c r="G99" t="inlineStr"/>
+        <v>2303.25</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -3122,7 +3084,7 @@
       <c r="B100" t="n">
         <v>1</v>
       </c>
-      <c r="C100" s="1" t="n">
+      <c r="C100" s="3" t="n">
         <v>45559</v>
       </c>
       <c r="D100" t="inlineStr">
@@ -3132,13 +3094,12 @@
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>FND-DROP 19"-24"</t>
+          <t>FND-DROP 13"-18"</t>
         </is>
       </c>
       <c r="F100" s="2" t="n">
-        <v>3432.5</v>
-      </c>
-      <c r="G100" t="inlineStr"/>
+        <v>2303.25</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -3149,7 +3110,7 @@
       <c r="B101" t="n">
         <v>1</v>
       </c>
-      <c r="C101" s="1" t="n">
+      <c r="C101" s="3" t="n">
         <v>45559</v>
       </c>
       <c r="D101" t="inlineStr">
@@ -3159,361 +3120,324 @@
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>FND-DROP 19"-24"</t>
+          <t>FND-DROP 13"-18"</t>
         </is>
       </c>
       <c r="F101" s="2" t="n">
-        <v>3432.5</v>
-      </c>
-      <c r="G101" t="inlineStr"/>
+        <v>2303.25</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>Edgewood</t>
-        </is>
-      </c>
-      <c r="B102" t="inlineStr">
-        <is>
-          <t>Landscape</t>
-        </is>
-      </c>
-      <c r="C102" s="1" t="n">
-        <v>45349</v>
+          <t>Edgewood - Concrete</t>
+        </is>
+      </c>
+      <c r="B102" t="n">
+        <v>1</v>
+      </c>
+      <c r="C102" s="3" t="n">
+        <v>45559</v>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>Typical Lot</t>
+          <t>Plan 1A</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>RG</t>
+          <t>FND-DROP 19"-24"</t>
         </is>
       </c>
       <c r="F102" s="2" t="n">
-        <v>450</v>
-      </c>
-      <c r="G102" t="inlineStr"/>
+        <v>3432.5</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>Edgewood</t>
-        </is>
-      </c>
-      <c r="B103" t="inlineStr">
-        <is>
-          <t>Landscape</t>
-        </is>
-      </c>
-      <c r="C103" s="1" t="n">
-        <v>45349</v>
+          <t>Edgewood - Concrete</t>
+        </is>
+      </c>
+      <c r="B103" t="n">
+        <v>1</v>
+      </c>
+      <c r="C103" s="3" t="n">
+        <v>45559</v>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>Typical Lot</t>
+          <t>Plan 1B</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>FG</t>
+          <t>FND-DROP 19"-24"</t>
         </is>
       </c>
       <c r="F103" s="2" t="n">
-        <v>375</v>
-      </c>
-      <c r="G103" t="inlineStr"/>
+        <v>3432.5</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>Edgewood</t>
-        </is>
-      </c>
-      <c r="B104" t="inlineStr">
-        <is>
-          <t>Landscape</t>
-        </is>
-      </c>
-      <c r="C104" s="1" t="n">
-        <v>45349</v>
+          <t>Edgewood - Concrete</t>
+        </is>
+      </c>
+      <c r="B104" t="n">
+        <v>1</v>
+      </c>
+      <c r="C104" s="3" t="n">
+        <v>45559</v>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>Typical Lot</t>
+          <t>Plan 1C</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>Irrigation</t>
+          <t>FND-DROP 19"-24"</t>
         </is>
       </c>
       <c r="F104" s="2" t="n">
-        <v>800</v>
-      </c>
-      <c r="G104" t="inlineStr"/>
+        <v>3432.5</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>Edgewood</t>
-        </is>
-      </c>
-      <c r="B105" t="inlineStr">
-        <is>
-          <t>Landscape</t>
-        </is>
-      </c>
-      <c r="C105" s="1" t="n">
-        <v>45349</v>
+          <t>Edgewood - Concrete</t>
+        </is>
+      </c>
+      <c r="B105" t="n">
+        <v>1</v>
+      </c>
+      <c r="C105" s="3" t="n">
+        <v>45559</v>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>Typical Lot</t>
+          <t>Plan 2A</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>LS</t>
+          <t>FND-DROP 19"-24"</t>
         </is>
       </c>
       <c r="F105" s="2" t="n">
-        <v>6449</v>
-      </c>
-      <c r="G105" t="inlineStr"/>
+        <v>3432.5</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>Edgewood</t>
-        </is>
-      </c>
-      <c r="B106" t="inlineStr">
-        <is>
-          <t>Landscape</t>
-        </is>
-      </c>
-      <c r="C106" s="1" t="n">
-        <v>45349</v>
+          <t>Edgewood - Concrete</t>
+        </is>
+      </c>
+      <c r="B106" t="n">
+        <v>1</v>
+      </c>
+      <c r="C106" s="3" t="n">
+        <v>45559</v>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>Typical Lot</t>
+          <t>Plan 2B</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>Haul Off (Rake-out/Spoil)</t>
+          <t>FND-DROP 19"-24"</t>
         </is>
       </c>
       <c r="F106" s="2" t="n">
-        <v>375</v>
-      </c>
-      <c r="G106" t="inlineStr"/>
+        <v>3432.5</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>Edgewood</t>
-        </is>
-      </c>
-      <c r="B107" t="inlineStr">
-        <is>
-          <t>Landscape</t>
-        </is>
-      </c>
-      <c r="C107" s="1" t="n">
-        <v>45349</v>
+          <t>Edgewood - Concrete</t>
+        </is>
+      </c>
+      <c r="B107" t="n">
+        <v>1</v>
+      </c>
+      <c r="C107" s="3" t="n">
+        <v>45559</v>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>Typical Lot</t>
+          <t>Plan 2C</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>AC Pipe Drainage</t>
+          <t>FND-DROP 19"-24"</t>
         </is>
       </c>
       <c r="F107" s="2" t="n">
-        <v>60</v>
-      </c>
-      <c r="G107" t="inlineStr"/>
+        <v>3432.5</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>Edgewood</t>
-        </is>
-      </c>
-      <c r="B108" t="inlineStr">
-        <is>
-          <t>Landscape</t>
-        </is>
-      </c>
-      <c r="C108" s="1" t="n">
-        <v>45349</v>
+          <t>Edgewood - Concrete</t>
+        </is>
+      </c>
+      <c r="B108" t="n">
+        <v>1</v>
+      </c>
+      <c r="C108" s="3" t="n">
+        <v>45559</v>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>Knuckle Lots 21 &amp; 43</t>
+          <t>Plan 3A</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>RG</t>
+          <t>FND-DROP 19"-24"</t>
         </is>
       </c>
       <c r="F108" s="2" t="n">
-        <v>450</v>
-      </c>
-      <c r="G108" t="inlineStr"/>
+        <v>3432.5</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>Edgewood</t>
-        </is>
-      </c>
-      <c r="B109" t="inlineStr">
-        <is>
-          <t>Landscape</t>
-        </is>
-      </c>
-      <c r="C109" s="1" t="n">
-        <v>45349</v>
+          <t>Edgewood - Concrete</t>
+        </is>
+      </c>
+      <c r="B109" t="n">
+        <v>1</v>
+      </c>
+      <c r="C109" s="3" t="n">
+        <v>45559</v>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>Knuckle Lots 21 &amp; 43</t>
+          <t>Plan 3B</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>FG</t>
+          <t>FND-DROP 19"-24"</t>
         </is>
       </c>
       <c r="F109" s="2" t="n">
-        <v>375</v>
-      </c>
-      <c r="G109" t="inlineStr"/>
+        <v>3432.5</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>Edgewood</t>
-        </is>
-      </c>
-      <c r="B110" t="inlineStr">
-        <is>
-          <t>Landscape</t>
-        </is>
-      </c>
-      <c r="C110" s="1" t="n">
-        <v>45349</v>
+          <t>Edgewood - Concrete</t>
+        </is>
+      </c>
+      <c r="B110" t="n">
+        <v>1</v>
+      </c>
+      <c r="C110" s="3" t="n">
+        <v>45559</v>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>Knuckle Lots 21 &amp; 43</t>
+          <t>Plan 3C</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>Irrigation</t>
+          <t>FND-DROP 19"-24"</t>
         </is>
       </c>
       <c r="F110" s="2" t="n">
-        <v>800</v>
-      </c>
-      <c r="G110" t="inlineStr"/>
+        <v>3432.5</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>Edgewood</t>
-        </is>
-      </c>
-      <c r="B111" t="inlineStr">
-        <is>
-          <t>Landscape</t>
-        </is>
-      </c>
-      <c r="C111" s="1" t="n">
-        <v>45349</v>
+          <t>Edgewood - Concrete</t>
+        </is>
+      </c>
+      <c r="B111" t="n">
+        <v>1</v>
+      </c>
+      <c r="C111" s="3" t="n">
+        <v>45559</v>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>Knuckle Lots 21 &amp; 43</t>
+          <t>Plan 4A</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>LS</t>
+          <t>FND-DROP 19"-24"</t>
         </is>
       </c>
       <c r="F111" s="2" t="n">
-        <v>8355</v>
-      </c>
-      <c r="G111" t="inlineStr"/>
+        <v>3432.5</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>Edgewood</t>
-        </is>
-      </c>
-      <c r="B112" t="inlineStr">
-        <is>
-          <t>Landscape</t>
-        </is>
-      </c>
-      <c r="C112" s="1" t="n">
-        <v>45349</v>
+          <t>Edgewood - Concrete</t>
+        </is>
+      </c>
+      <c r="B112" t="n">
+        <v>1</v>
+      </c>
+      <c r="C112" s="3" t="n">
+        <v>45559</v>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>Knuckle Lots 21 &amp; 43</t>
+          <t>Plan 4B</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>Haul Off (Rake-out/Spoil)</t>
+          <t>FND-DROP 19"-24"</t>
         </is>
       </c>
       <c r="F112" s="2" t="n">
-        <v>375</v>
-      </c>
-      <c r="G112" t="inlineStr"/>
+        <v>3432.5</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>Edgewood</t>
-        </is>
-      </c>
-      <c r="B113" t="inlineStr">
-        <is>
-          <t>Landscape</t>
-        </is>
-      </c>
-      <c r="C113" s="1" t="n">
-        <v>45349</v>
+          <t>Edgewood - Concrete</t>
+        </is>
+      </c>
+      <c r="B113" t="n">
+        <v>1</v>
+      </c>
+      <c r="C113" s="3" t="n">
+        <v>45559</v>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>Knuckle Lots 21 &amp; 43</t>
+          <t>Plan 4C</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>AC Pipe Drainage</t>
+          <t>FND-DROP 19"-24"</t>
         </is>
       </c>
       <c r="F113" s="2" t="n">
-        <v>60</v>
-      </c>
-      <c r="G113" t="inlineStr"/>
+        <v>3432.5</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -3526,12 +3450,12 @@
           <t>Landscape</t>
         </is>
       </c>
-      <c r="C114" s="1" t="n">
+      <c r="C114" s="3" t="n">
         <v>45349</v>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>Oversized Lots 17 &amp; 18</t>
+          <t>Typical Lot</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
@@ -3542,7 +3466,6 @@
       <c r="F114" s="2" t="n">
         <v>450</v>
       </c>
-      <c r="G114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -3555,12 +3478,12 @@
           <t>Landscape</t>
         </is>
       </c>
-      <c r="C115" s="1" t="n">
+      <c r="C115" s="3" t="n">
         <v>45349</v>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>Oversized Lots 17 &amp; 18</t>
+          <t>Typical Lot</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
@@ -3571,7 +3494,6 @@
       <c r="F115" s="2" t="n">
         <v>375</v>
       </c>
-      <c r="G115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -3584,12 +3506,12 @@
           <t>Landscape</t>
         </is>
       </c>
-      <c r="C116" s="1" t="n">
+      <c r="C116" s="3" t="n">
         <v>45349</v>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>Oversized Lots 17 &amp; 18</t>
+          <t>Typical Lot</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
@@ -3600,7 +3522,6 @@
       <c r="F116" s="2" t="n">
         <v>800</v>
       </c>
-      <c r="G116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -3613,12 +3534,12 @@
           <t>Landscape</t>
         </is>
       </c>
-      <c r="C117" s="1" t="n">
+      <c r="C117" s="3" t="n">
         <v>45349</v>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>Oversized Lots 17 &amp; 18</t>
+          <t>Typical Lot</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
@@ -3627,9 +3548,8 @@
         </is>
       </c>
       <c r="F117" s="2" t="n">
-        <v>5025</v>
-      </c>
-      <c r="G117" t="inlineStr"/>
+        <v>6449</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -3642,12 +3562,12 @@
           <t>Landscape</t>
         </is>
       </c>
-      <c r="C118" s="1" t="n">
+      <c r="C118" s="3" t="n">
         <v>45349</v>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>Oversized Lots 17 &amp; 18</t>
+          <t>Typical Lot</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
@@ -3658,7 +3578,6 @@
       <c r="F118" s="2" t="n">
         <v>375</v>
       </c>
-      <c r="G118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -3671,12 +3590,12 @@
           <t>Landscape</t>
         </is>
       </c>
-      <c r="C119" s="1" t="n">
+      <c r="C119" s="3" t="n">
         <v>45349</v>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>Oversized Lots 17 &amp; 18</t>
+          <t>Typical Lot</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
@@ -3687,7 +3606,6 @@
       <c r="F119" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="G119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -3697,26 +3615,25 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>Pavers</t>
-        </is>
-      </c>
-      <c r="C120" s="1" t="n">
+          <t>Landscape</t>
+        </is>
+      </c>
+      <c r="C120" s="3" t="n">
         <v>45349</v>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>Plan 1ABC</t>
+          <t>Knuckle Lots 21 &amp; 43</t>
         </is>
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>Pavers</t>
+          <t>RG</t>
         </is>
       </c>
       <c r="F120" s="2" t="n">
-        <v>3479</v>
-      </c>
-      <c r="G120" t="inlineStr"/>
+        <v>450</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -3726,26 +3643,25 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>Pavers</t>
-        </is>
-      </c>
-      <c r="C121" s="1" t="n">
+          <t>Landscape</t>
+        </is>
+      </c>
+      <c r="C121" s="3" t="n">
         <v>45349</v>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>Plan 2ABC</t>
+          <t>Knuckle Lots 21 &amp; 43</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>Pavers</t>
+          <t>FG</t>
         </is>
       </c>
       <c r="F121" s="2" t="n">
-        <v>3675</v>
-      </c>
-      <c r="G121" t="inlineStr"/>
+        <v>375</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -3755,26 +3671,25 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>Pavers</t>
-        </is>
-      </c>
-      <c r="C122" s="1" t="n">
+          <t>Landscape</t>
+        </is>
+      </c>
+      <c r="C122" s="3" t="n">
         <v>45349</v>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>Plan 3ABC</t>
+          <t>Knuckle Lots 21 &amp; 43</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>Pavers</t>
+          <t>Irrigation</t>
         </is>
       </c>
       <c r="F122" s="2" t="n">
-        <v>2671</v>
-      </c>
-      <c r="G122" t="inlineStr"/>
+        <v>800</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -3784,26 +3699,25 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>Pavers</t>
-        </is>
-      </c>
-      <c r="C123" s="1" t="n">
+          <t>Landscape</t>
+        </is>
+      </c>
+      <c r="C123" s="3" t="n">
         <v>45349</v>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>Plan 4ABC</t>
+          <t>Knuckle Lots 21 &amp; 43</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>Pavers</t>
+          <t>LS</t>
         </is>
       </c>
       <c r="F123" s="2" t="n">
-        <v>2377</v>
-      </c>
-      <c r="G123" t="inlineStr"/>
+        <v>8355</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -3813,26 +3727,25 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>Pavers</t>
-        </is>
-      </c>
-      <c r="C124" s="1" t="n">
-        <v>45775</v>
+          <t>Landscape</t>
+        </is>
+      </c>
+      <c r="C124" s="3" t="n">
+        <v>45349</v>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>Plan 1ABC</t>
+          <t>Knuckle Lots 21 &amp; 43</t>
         </is>
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>Pavers</t>
+          <t>Haul Off (Rake-out/Spoil)</t>
         </is>
       </c>
       <c r="F124" s="2" t="n">
-        <v>3834</v>
-      </c>
-      <c r="G124" t="inlineStr"/>
+        <v>375</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -3842,26 +3755,25 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>Pavers</t>
-        </is>
-      </c>
-      <c r="C125" s="1" t="n">
-        <v>45775</v>
+          <t>Landscape</t>
+        </is>
+      </c>
+      <c r="C125" s="3" t="n">
+        <v>45349</v>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>Plan 2ABC</t>
+          <t>Knuckle Lots 21 &amp; 43</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>Pavers</t>
+          <t>AC Pipe Drainage</t>
         </is>
       </c>
       <c r="F125" s="2" t="n">
-        <v>4030</v>
-      </c>
-      <c r="G125" t="inlineStr"/>
+        <v>60</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -3871,26 +3783,25 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>Pavers</t>
-        </is>
-      </c>
-      <c r="C126" s="1" t="n">
-        <v>45775</v>
+          <t>Landscape</t>
+        </is>
+      </c>
+      <c r="C126" s="3" t="n">
+        <v>45349</v>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>Plan 3ABC</t>
+          <t>Oversized Lots 17 &amp; 18</t>
         </is>
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>Pavers</t>
+          <t>RG</t>
         </is>
       </c>
       <c r="F126" s="2" t="n">
-        <v>2707</v>
-      </c>
-      <c r="G126" t="inlineStr"/>
+        <v>450</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -3900,26 +3811,361 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
+          <t>Landscape</t>
+        </is>
+      </c>
+      <c r="C127" s="3" t="n">
+        <v>45349</v>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>Oversized Lots 17 &amp; 18</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>FG</t>
+        </is>
+      </c>
+      <c r="F127" s="2" t="n">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>Edgewood</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>Landscape</t>
+        </is>
+      </c>
+      <c r="C128" s="3" t="n">
+        <v>45349</v>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>Oversized Lots 17 &amp; 18</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>Irrigation</t>
+        </is>
+      </c>
+      <c r="F128" s="2" t="n">
+        <v>800</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>Edgewood</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>Landscape</t>
+        </is>
+      </c>
+      <c r="C129" s="3" t="n">
+        <v>45349</v>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>Oversized Lots 17 &amp; 18</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>LS</t>
+        </is>
+      </c>
+      <c r="F129" s="2" t="n">
+        <v>5025</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>Edgewood</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>Landscape</t>
+        </is>
+      </c>
+      <c r="C130" s="3" t="n">
+        <v>45349</v>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>Oversized Lots 17 &amp; 18</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>Haul Off (Rake-out/Spoil)</t>
+        </is>
+      </c>
+      <c r="F130" s="2" t="n">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>Edgewood</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>Landscape</t>
+        </is>
+      </c>
+      <c r="C131" s="3" t="n">
+        <v>45349</v>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>Oversized Lots 17 &amp; 18</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>AC Pipe Drainage</t>
+        </is>
+      </c>
+      <c r="F131" s="2" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>Edgewood</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
           <t>Pavers</t>
         </is>
       </c>
-      <c r="C127" s="1" t="n">
+      <c r="C132" s="3" t="n">
+        <v>45349</v>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>Plan 1ABC</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>Pavers</t>
+        </is>
+      </c>
+      <c r="F132" s="2" t="n">
+        <v>3479</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>Edgewood</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>Pavers</t>
+        </is>
+      </c>
+      <c r="C133" s="3" t="n">
+        <v>45349</v>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>Plan 2ABC</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>Pavers</t>
+        </is>
+      </c>
+      <c r="F133" s="2" t="n">
+        <v>3675</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>Edgewood</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>Pavers</t>
+        </is>
+      </c>
+      <c r="C134" s="3" t="n">
+        <v>45349</v>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>Plan 3ABC</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>Pavers</t>
+        </is>
+      </c>
+      <c r="F134" s="2" t="n">
+        <v>2671</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>Edgewood</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>Pavers</t>
+        </is>
+      </c>
+      <c r="C135" s="3" t="n">
+        <v>45349</v>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>Plan 4ABC</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>Pavers</t>
+        </is>
+      </c>
+      <c r="F135" s="2" t="n">
+        <v>2377</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>Edgewood</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>Pavers</t>
+        </is>
+      </c>
+      <c r="C136" s="3" t="n">
         <v>45775</v>
       </c>
-      <c r="D127" t="inlineStr">
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>Plan 1ABC</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>Pavers</t>
+        </is>
+      </c>
+      <c r="F136" s="2" t="n">
+        <v>3834</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>Edgewood</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>Pavers</t>
+        </is>
+      </c>
+      <c r="C137" s="3" t="n">
+        <v>45775</v>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>Plan 2ABC</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>Pavers</t>
+        </is>
+      </c>
+      <c r="F137" s="2" t="n">
+        <v>4030</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>Edgewood</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>Pavers</t>
+        </is>
+      </c>
+      <c r="C138" s="3" t="n">
+        <v>45775</v>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>Plan 3ABC</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>Pavers</t>
+        </is>
+      </c>
+      <c r="F138" s="2" t="n">
+        <v>2707</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>Edgewood</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>Pavers</t>
+        </is>
+      </c>
+      <c r="C139" s="3" t="n">
+        <v>45775</v>
+      </c>
+      <c r="D139" t="inlineStr">
         <is>
           <t>Plan 4ABC</t>
         </is>
       </c>
-      <c r="E127" t="inlineStr">
+      <c r="E139" t="inlineStr">
         <is>
           <t>Pavers</t>
         </is>
       </c>
-      <c r="F127" s="2" t="n">
+      <c r="F139" s="2" t="n">
         <v>2413</v>
       </c>
-      <c r="G127" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>